<commit_message>
fix: correct 15-digit NIKs in RW 6 and RW 7 Excel files, regenerate dpt_seed.csv, and add strict 16-digit validation to bangun_dpt_seed.py
</commit_message>
<xml_diff>
--- a/DPS PILKADES 2026/RW 6.xlsx
+++ b/DPS PILKADES 2026/RW 6.xlsx
@@ -9510,7 +9510,7 @@
       </c>
       <c r="U124" s="81" t="inlineStr">
         <is>
-          <t>610301110795001</t>
+          <t>6103011107950001</t>
         </is>
       </c>
       <c r="V124" s="81" t="inlineStr">
@@ -34704,7 +34704,7 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="B4:S4"/>
+    <mergeCell ref="L7:R7"/>
     <mergeCell ref="B3:S3"/>
     <mergeCell ref="B2:S2"/>
     <mergeCell ref="C7:C8"/>
@@ -34718,9 +34718,9 @@
     <mergeCell ref="G7:G8"/>
     <mergeCell ref="H7:H8"/>
     <mergeCell ref="I7:I8"/>
+    <mergeCell ref="B4:S4"/>
     <mergeCell ref="J7:J8"/>
     <mergeCell ref="K7:K8"/>
-    <mergeCell ref="L7:R7"/>
     <mergeCell ref="U7:U8"/>
   </mergeCells>
   <pageMargins left="0.7874015748031497" right="0.3937007874015748" top="0.3937007874015748" bottom="0.3937007874015748" header="0.3149606299212598" footer="0.3149606299212598"/>
@@ -34743,7 +34743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S32"/>
+  <dimension ref="A6:S32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.90625" defaultRowHeight="15"/>
   <cols>
     <col width="5.1796875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -34758,10 +34758,6 @@
     <col width="2.1796875" bestFit="1" customWidth="1" min="13" max="19"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="15.6" customHeight="1" thickBot="1"/>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
@@ -35946,8 +35942,9 @@
   <mergeCells count="14">
     <mergeCell ref="M6:S6"/>
     <mergeCell ref="C7:C8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="G7:G8"/>
     <mergeCell ref="M7:S7"/>
-    <mergeCell ref="G7:G8"/>
     <mergeCell ref="E7:E8"/>
     <mergeCell ref="A7:A8"/>
     <mergeCell ref="K7:K8"/>
@@ -35955,7 +35952,6 @@
     <mergeCell ref="F7:F8"/>
     <mergeCell ref="J7:J8"/>
     <mergeCell ref="I7:I8"/>
-    <mergeCell ref="B7:B8"/>
     <mergeCell ref="L7:L8"/>
     <mergeCell ref="D7:D8"/>
   </mergeCells>
@@ -35969,7 +35965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S19"/>
+  <dimension ref="A6:S19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.90625" defaultRowHeight="15"/>
   <cols>
     <col width="5.1796875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -35984,10 +35980,6 @@
     <col width="2.1796875" bestFit="1" customWidth="1" min="13" max="19"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="15.6" customHeight="1" thickBot="1"/>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
@@ -36715,8 +36707,9 @@
   <mergeCells count="14">
     <mergeCell ref="M6:S6"/>
     <mergeCell ref="C7:C8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="G7:G8"/>
     <mergeCell ref="M7:S7"/>
-    <mergeCell ref="G7:G8"/>
     <mergeCell ref="E7:E8"/>
     <mergeCell ref="A7:A8"/>
     <mergeCell ref="K7:K8"/>
@@ -36724,7 +36717,6 @@
     <mergeCell ref="F7:F8"/>
     <mergeCell ref="J7:J8"/>
     <mergeCell ref="I7:I8"/>
-    <mergeCell ref="B7:B8"/>
     <mergeCell ref="L7:L8"/>
     <mergeCell ref="D7:D8"/>
   </mergeCells>
@@ -36740,9 +36732,7 @@
   </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1"/>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -36755,9 +36745,7 @@
   </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1"/>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -36768,7 +36756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S125"/>
+  <dimension ref="A6:S125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.1796875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -36784,10 +36772,6 @@
     <col width="2.1796875" bestFit="1" customWidth="1" min="13" max="19"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="15.6" customHeight="1" thickBot="1"/>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
@@ -43524,8 +43508,8 @@
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="M7:S7"/>
     <mergeCell ref="G7:G8"/>
+    <mergeCell ref="B7:B8"/>
     <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
     <mergeCell ref="D7:D8"/>
     <mergeCell ref="I7:I8"/>
     <mergeCell ref="M6:S6"/>
@@ -43546,7 +43530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S43"/>
+  <dimension ref="A6:S43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.1796875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -43562,10 +43546,6 @@
     <col width="2.1796875" bestFit="1" customWidth="1" min="13" max="19"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="15.6" customHeight="1" thickBot="1"/>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
@@ -45714,8 +45694,8 @@
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="M7:S7"/>
     <mergeCell ref="G7:G8"/>
+    <mergeCell ref="B7:B8"/>
     <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
     <mergeCell ref="D7:D8"/>
     <mergeCell ref="I7:I8"/>
     <mergeCell ref="M6:S6"/>
@@ -45736,7 +45716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S86"/>
+  <dimension ref="A6:S86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.1796875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -45752,10 +45732,6 @@
     <col width="2.1796875" bestFit="1" customWidth="1" min="13" max="19"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="15.6" customHeight="1" thickBot="1"/>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
@@ -50223,8 +50199,8 @@
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="M7:S7"/>
     <mergeCell ref="G7:G8"/>
+    <mergeCell ref="B7:B8"/>
     <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
     <mergeCell ref="D7:D8"/>
     <mergeCell ref="I7:I8"/>
     <mergeCell ref="M6:S6"/>
@@ -50245,7 +50221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S80"/>
+  <dimension ref="A6:S80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.1796875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -50261,10 +50237,6 @@
     <col width="2.1796875" bestFit="1" customWidth="1" min="13" max="19"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="15.6" customHeight="1" thickBot="1"/>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
@@ -54514,7 +54486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S57"/>
+  <dimension ref="A6:S57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.1796875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -54530,10 +54502,6 @@
     <col width="2.1796875" bestFit="1" customWidth="1" min="13" max="19"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="15.6" customHeight="1" thickBot="1"/>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
@@ -57424,8 +57392,8 @@
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="M7:S7"/>
     <mergeCell ref="G7:G8"/>
+    <mergeCell ref="B7:B8"/>
     <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
     <mergeCell ref="D7:D8"/>
     <mergeCell ref="I7:I8"/>
     <mergeCell ref="M6:S6"/>
@@ -57446,7 +57414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S21"/>
+  <dimension ref="A6:S21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.1796875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -57462,10 +57430,6 @@
     <col width="2.1796875" bestFit="1" customWidth="1" min="13" max="19"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="15.6" customHeight="1" thickBot="1"/>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
@@ -58360,8 +58324,8 @@
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="M7:S7"/>
     <mergeCell ref="G7:G8"/>
+    <mergeCell ref="B7:B8"/>
     <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
     <mergeCell ref="D7:D8"/>
     <mergeCell ref="I7:I8"/>
     <mergeCell ref="M6:S6"/>
@@ -58382,7 +58346,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S35"/>
+  <dimension ref="A6:S35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.1796875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -58398,10 +58362,6 @@
     <col width="2.1796875" bestFit="1" customWidth="1" min="13" max="19"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="15.6" customHeight="1" thickBot="1"/>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
@@ -60094,8 +60054,8 @@
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="M7:S7"/>
     <mergeCell ref="G7:G8"/>
+    <mergeCell ref="B7:B8"/>
     <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
     <mergeCell ref="D7:D8"/>
     <mergeCell ref="I7:I8"/>
     <mergeCell ref="M6:S6"/>
@@ -60116,7 +60076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S97"/>
+  <dimension ref="A6:S97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.1796875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -60132,10 +60092,6 @@
     <col width="2.1796875" bestFit="1" customWidth="1" min="13" max="19"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="15.6" customHeight="1" thickBot="1"/>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
@@ -65306,8 +65262,8 @@
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="M7:S7"/>
     <mergeCell ref="G7:G8"/>
+    <mergeCell ref="B7:B8"/>
     <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
     <mergeCell ref="D7:D8"/>
     <mergeCell ref="I7:I8"/>
     <mergeCell ref="M6:S6"/>

</xml_diff>